<commit_message>
Exclui fornecedor 789429 da apuracao de gerentes e atualiza metas
As vendas da Prati Donaduzzi (789429) deixam de contar apenas na aba de
Gerentes; demais abas seguem com o pedido total. Atualiza as planilhas de
meta de fornecedor/filial, gerente e supervisor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/meta fornecedor filial.xlsx
+++ b/data/meta fornecedor filial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F906F1A-6323-438B-A048-95BE9BF25AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05215801-2957-44D9-B63D-E3BF7E95C63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{669ECB6C-83CF-4053-B745-2A03E06ED1EB}"/>
   </bookViews>
@@ -815,7 +815,7 @@
         <v>21</v>
       </c>
       <c r="E2">
-        <v>262965.12</v>
+        <v>262965.15999999997</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>